<commit_message>
chore(db): reset data + refactor essais_* pipeline & consolidated views
- Migrations 026-028: AMESSEFE preparation, essais_classif unification, consolidated views
- Migration 027b: add echantillon_id to essais_physiques
- Refactor 02_import_excel.py: write to essais_classif, essais_physiques (not essais_geotechniques)
- Refactor 03_import_amessefe.py: write to essais_vbs, essais_classif, granulo_points
- Create atlas.v_echantillons_essais: consolidated view joining all essais_* tables
- Harmonize laboratory='FORMATEC' across all echantillons
- Architecture: essais_* tables = source of truth, views = aggregation layer
</commit_message>
<xml_diff>
--- a/data/xlsx/IMPORT/atlas_import_nicabou_ninsao_vianney.xlsx
+++ b/data/xlsx/IMPORT/atlas_import_nicabou_ninsao_vianney.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROJET_ATLAS_MASTER\atlas\data\xlsx\IMPORT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP EITEBOOK\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C29778B-9329-4A7C-AB9E-BDE6E90BEAB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3CADB6E-41D1-453A-B288-1991219264FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="agt_raw_long" sheetId="3" r:id="rId1"/>
@@ -26,12 +26,28 @@
     <sheet name="echantillons" sheetId="15" r:id="rId11"/>
     <sheet name="meta" sheetId="17" r:id="rId12"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="71">
   <si>
     <t>sieve_mm</t>
   </si>
@@ -129,9 +145,6 @@
     <t>DAVIE@2.0</t>
   </si>
   <si>
-    <t>DAVIE</t>
-  </si>
-  <si>
     <t>wl</t>
   </si>
   <si>
@@ -207,9 +220,6 @@
     <t>NICABOU Ninsao Vianney</t>
   </si>
   <si>
-    <t>Davie</t>
-  </si>
-  <si>
     <t>Dzogbecope</t>
   </si>
   <si>
@@ -244,6 +254,12 @@
   </si>
   <si>
     <t>Import structuré depuis données brutes (partie 1)</t>
+  </si>
+  <si>
+    <t>ZIO</t>
+  </si>
+  <si>
+    <t>FORMATEC</t>
   </si>
 </sst>
 </file>
@@ -302,11 +318,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -325,9 +342,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -365,9 +382,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -400,26 +417,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -452,26 +452,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -646,9 +629,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F163"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.7265625" customWidth="1"/>
+    <col min="5" max="5" width="22.7265625" customWidth="1"/>
+    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -668,7 +659,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -682,7 +673,7 @@
         <v>10.76</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -696,7 +687,7 @@
         <v>12.22</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -710,7 +701,7 @@
         <v>13.69</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -724,7 +715,7 @@
         <v>15.16</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -738,7 +729,7 @@
         <v>17.600000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -752,7 +743,7 @@
         <v>21.03</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -766,7 +757,7 @@
         <v>24.94</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -780,7 +771,7 @@
         <v>28.85</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -794,7 +785,7 @@
         <v>31.29</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -814,7 +805,7 @@
         <v>37.99</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -834,7 +825,7 @@
         <v>47.18</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -854,7 +845,7 @@
         <v>65.010000000000005</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -874,7 +865,7 @@
         <v>84.73</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -894,7 +885,7 @@
         <v>92.36</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>12</v>
       </c>
@@ -914,7 +905,7 @@
         <v>93.73</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>12</v>
       </c>
@@ -934,7 +925,7 @@
         <v>95.23</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>12</v>
       </c>
@@ -954,7 +945,7 @@
         <v>99.4</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>12</v>
       </c>
@@ -974,7 +965,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -994,7 +985,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>12</v>
       </c>
@@ -1014,7 +1005,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>12</v>
       </c>
@@ -1028,7 +1019,7 @@
         <v>31.45</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>12</v>
       </c>
@@ -1042,7 +1033,7 @@
         <v>33.229999999999997</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>12</v>
       </c>
@@ -1056,7 +1047,7 @@
         <v>36.450000000000003</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -1070,7 +1061,7 @@
         <v>39.03</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>12</v>
       </c>
@@ -1084,7 +1075,7 @@
         <v>41.45</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>12</v>
       </c>
@@ -1098,7 +1089,7 @@
         <v>44.35</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>12</v>
       </c>
@@ -1112,7 +1103,7 @@
         <v>46.77</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>12</v>
       </c>
@@ -1132,7 +1123,7 @@
         <v>50.58</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>12</v>
       </c>
@@ -1152,7 +1143,7 @@
         <v>58.41</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>12</v>
       </c>
@@ -1172,7 +1163,7 @@
         <v>75.09</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>12</v>
       </c>
@@ -1192,7 +1183,7 @@
         <v>91.51</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>12</v>
       </c>
@@ -1212,7 +1203,7 @@
         <v>98.82</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>12</v>
       </c>
@@ -1232,7 +1223,7 @@
         <v>99.87</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>12</v>
       </c>
@@ -1252,7 +1243,7 @@
         <v>99.97</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>12</v>
       </c>
@@ -1272,7 +1263,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>12</v>
       </c>
@@ -1292,7 +1283,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>12</v>
       </c>
@@ -1312,7 +1303,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>12</v>
       </c>
@@ -1332,7 +1323,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>12</v>
       </c>
@@ -1346,7 +1337,7 @@
         <v>33.369999999999997</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>12</v>
       </c>
@@ -1360,7 +1351,7 @@
         <v>36.97</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>12</v>
       </c>
@@ -1374,7 +1365,7 @@
         <v>40.58</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>12</v>
       </c>
@@ -1388,7 +1379,7 @@
         <v>43.23</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>12</v>
       </c>
@@ -1402,7 +1393,7 @@
         <v>45.09</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>12</v>
       </c>
@@ -1422,7 +1413,7 @@
         <v>50.24</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>12</v>
       </c>
@@ -1442,7 +1433,7 @@
         <v>58.74</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>12</v>
       </c>
@@ -1462,7 +1453,7 @@
         <v>75.180000000000007</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>12</v>
       </c>
@@ -1482,7 +1473,7 @@
         <v>91.68</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>12</v>
       </c>
@@ -1502,7 +1493,7 @@
         <v>98.85</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>12</v>
       </c>
@@ -1522,7 +1513,7 @@
         <v>99.92</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>12</v>
       </c>
@@ -1542,7 +1533,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>12</v>
       </c>
@@ -1562,7 +1553,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>12</v>
       </c>
@@ -1582,7 +1573,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>12</v>
       </c>
@@ -1602,7 +1593,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>12</v>
       </c>
@@ -1622,7 +1613,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>13</v>
       </c>
@@ -1636,7 +1627,7 @@
         <v>21.68</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>13</v>
       </c>
@@ -1650,7 +1641,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>13</v>
       </c>
@@ -1664,7 +1655,7 @@
         <v>27.64</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>13</v>
       </c>
@@ -1678,7 +1669,7 @@
         <v>32.01</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>13</v>
       </c>
@@ -1692,7 +1683,7 @@
         <v>36.369999999999997</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>13</v>
       </c>
@@ -1706,7 +1697,7 @@
         <v>40.01</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>13</v>
       </c>
@@ -1720,7 +1711,7 @@
         <v>42.82</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>13</v>
       </c>
@@ -1740,7 +1731,7 @@
         <v>47.9</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>13</v>
       </c>
@@ -1760,7 +1751,7 @@
         <v>58.7</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>13</v>
       </c>
@@ -1780,7 +1771,7 @@
         <v>76.510000000000005</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>13</v>
       </c>
@@ -1800,7 +1791,7 @@
         <v>91.43</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>13</v>
       </c>
@@ -1820,7 +1811,7 @@
         <v>97.4</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>13</v>
       </c>
@@ -1840,7 +1831,7 @@
         <v>98.43</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>13</v>
       </c>
@@ -1860,7 +1851,7 @@
         <v>98.9</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>13</v>
       </c>
@@ -1874,7 +1865,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>13</v>
       </c>
@@ -1888,7 +1879,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>13</v>
       </c>
@@ -1902,7 +1893,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>13</v>
       </c>
@@ -1916,7 +1907,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>13</v>
       </c>
@@ -1930,7 +1921,7 @@
         <v>21.82</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>13</v>
       </c>
@@ -1944,7 +1935,7 @@
         <v>25.6</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>13</v>
       </c>
@@ -1958,7 +1949,7 @@
         <v>32.729999999999997</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>13</v>
       </c>
@@ -1972,7 +1963,7 @@
         <v>37.85</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>13</v>
       </c>
@@ -1986,7 +1977,7 @@
         <v>42.08</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>13</v>
       </c>
@@ -2000,7 +1991,7 @@
         <v>45.64</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>13</v>
       </c>
@@ -2014,7 +2005,7 @@
         <v>48.98</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>13</v>
       </c>
@@ -2034,7 +2025,7 @@
         <v>55.02</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>13</v>
       </c>
@@ -2054,7 +2045,7 @@
         <v>65.41</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>13</v>
       </c>
@@ -2074,7 +2065,7 @@
         <v>82.14</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>13</v>
       </c>
@@ -2094,7 +2085,7 @@
         <v>84.92</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>13</v>
       </c>
@@ -2114,7 +2105,7 @@
         <v>99.04</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>13</v>
       </c>
@@ -2134,7 +2125,7 @@
         <v>99.7</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>13</v>
       </c>
@@ -2154,7 +2145,7 @@
         <v>99.8</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>13</v>
       </c>
@@ -2168,7 +2159,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>13</v>
       </c>
@@ -2182,7 +2173,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>13</v>
       </c>
@@ -2196,7 +2187,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>13</v>
       </c>
@@ -2210,7 +2201,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>13</v>
       </c>
@@ -2224,7 +2215,7 @@
         <v>38.18</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>13</v>
       </c>
@@ -2238,7 +2229,7 @@
         <v>41.2</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>13</v>
       </c>
@@ -2252,7 +2243,7 @@
         <v>46.22</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>13</v>
       </c>
@@ -2266,7 +2257,7 @@
         <v>48.83</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>13</v>
       </c>
@@ -2280,7 +2271,7 @@
         <v>52.25</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>13</v>
       </c>
@@ -2294,7 +2285,7 @@
         <v>56.27</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>13</v>
       </c>
@@ -2308,7 +2299,7 @@
         <v>59.28</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>13</v>
       </c>
@@ -2328,7 +2319,7 @@
         <v>62.89</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>13</v>
       </c>
@@ -2348,7 +2339,7 @@
         <v>71.569999999999993</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>13</v>
       </c>
@@ -2368,7 +2359,7 @@
         <v>84.77</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>13</v>
       </c>
@@ -2388,7 +2379,7 @@
         <v>95.03</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>13</v>
       </c>
@@ -2408,7 +2399,7 @@
         <v>98.43</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>13</v>
       </c>
@@ -2428,7 +2419,7 @@
         <v>99.3</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>13</v>
       </c>
@@ -2448,7 +2439,7 @@
         <v>99.52</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>13</v>
       </c>
@@ -2462,7 +2453,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>13</v>
       </c>
@@ -2476,7 +2467,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>13</v>
       </c>
@@ -2490,7 +2481,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>13</v>
       </c>
@@ -2504,7 +2495,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>14</v>
       </c>
@@ -2518,7 +2509,7 @@
         <v>30.71</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>14</v>
       </c>
@@ -2532,7 +2523,7 @@
         <v>31.91</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>14</v>
       </c>
@@ -2546,7 +2537,7 @@
         <v>33.700000000000003</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>14</v>
       </c>
@@ -2560,7 +2551,7 @@
         <v>35.76</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>14</v>
       </c>
@@ -2574,7 +2565,7 @@
         <v>37.82</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>14</v>
       </c>
@@ -2588,7 +2579,7 @@
         <v>39.47</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>14</v>
       </c>
@@ -2602,7 +2593,7 @@
         <v>40.57</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>14</v>
       </c>
@@ -2622,7 +2613,7 @@
         <v>45.89</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>14</v>
       </c>
@@ -2642,7 +2633,7 @@
         <v>52.24</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>14</v>
       </c>
@@ -2662,7 +2653,7 @@
         <v>71.64</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>14</v>
       </c>
@@ -2682,7 +2673,7 @@
         <v>91.92</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>14</v>
       </c>
@@ -2702,7 +2693,7 @@
         <v>99.48</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>14</v>
       </c>
@@ -2722,7 +2713,7 @@
         <v>99.93</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>14</v>
       </c>
@@ -2736,7 +2727,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>14</v>
       </c>
@@ -2750,7 +2741,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>14</v>
       </c>
@@ -2764,7 +2755,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>14</v>
       </c>
@@ -2778,7 +2769,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>14</v>
       </c>
@@ -2792,7 +2783,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>14</v>
       </c>
@@ -2806,7 +2797,7 @@
         <v>26.56</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>14</v>
       </c>
@@ -2820,7 +2811,7 @@
         <v>27.99</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>14</v>
       </c>
@@ -2834,7 +2825,7 @@
         <v>30.41</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>14</v>
       </c>
@@ -2848,7 +2839,7 @@
         <v>33.409999999999997</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>14</v>
       </c>
@@ -2862,7 +2853,7 @@
         <v>36.409999999999997</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>14</v>
       </c>
@@ -2876,7 +2867,7 @@
         <v>38.979999999999997</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>14</v>
       </c>
@@ -2890,7 +2881,7 @@
         <v>41.27</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>14</v>
       </c>
@@ -2910,7 +2901,7 @@
         <v>44.68</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>14</v>
       </c>
@@ -2930,7 +2921,7 @@
         <v>51.32</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>14</v>
       </c>
@@ -2950,7 +2941,7 @@
         <v>71.53</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>14</v>
       </c>
@@ -2970,7 +2961,7 @@
         <v>92.58</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>14</v>
       </c>
@@ -2990,7 +2981,7 @@
         <v>99.6</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>14</v>
       </c>
@@ -3004,7 +2995,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>14</v>
       </c>
@@ -3018,7 +3009,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>14</v>
       </c>
@@ -3032,7 +3023,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>14</v>
       </c>
@@ -3046,7 +3037,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>14</v>
       </c>
@@ -3060,7 +3051,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>14</v>
       </c>
@@ -3074,7 +3065,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>14</v>
       </c>
@@ -3088,7 +3079,7 @@
         <v>26.33</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>14</v>
       </c>
@@ -3102,7 +3093,7 @@
         <v>28.28</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>14</v>
       </c>
@@ -3116,7 +3107,7 @@
         <v>32.18</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>14</v>
       </c>
@@ -3130,7 +3121,7 @@
         <v>37.06</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>14</v>
       </c>
@@ -3144,7 +3135,7 @@
         <v>42.33</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>14</v>
       </c>
@@ -3158,7 +3149,7 @@
         <v>46.62</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>14</v>
       </c>
@@ -3172,7 +3163,7 @@
         <v>49.54</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>14</v>
       </c>
@@ -3192,7 +3183,7 @@
         <v>53.1</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>14</v>
       </c>
@@ -3212,7 +3203,7 @@
         <v>58.95</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>14</v>
       </c>
@@ -3232,7 +3223,7 @@
         <v>75.19</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>14</v>
       </c>
@@ -3252,7 +3243,7 @@
         <v>93.1</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>14</v>
       </c>
@@ -3272,7 +3263,7 @@
         <v>99.53</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>14</v>
       </c>
@@ -3292,7 +3283,7 @@
         <v>99.99</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>14</v>
       </c>
@@ -3306,7 +3297,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>14</v>
       </c>
@@ -3320,7 +3311,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>14</v>
       </c>
@@ -3334,7 +3325,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>14</v>
       </c>
@@ -3348,7 +3339,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>14</v>
       </c>
@@ -3369,80 +3360,92 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{129F5F88-9951-44A9-9DEF-0F28384A941A}">
-  <dimension ref="A1:I5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="2" max="2" width="11.54296875" customWidth="1"/>
+    <col min="4" max="4" width="23.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="I1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C2" s="2">
+        <v>44531</v>
+      </c>
+      <c r="D2" t="s">
         <v>56</v>
       </c>
-      <c r="D2" t="s">
+      <c r="I2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C3" s="2">
+        <v>44531</v>
+      </c>
+      <c r="D3" t="s">
+        <v>56</v>
+      </c>
+      <c r="I3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
         <v>58</v>
       </c>
-      <c r="D3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
-        <v>59</v>
+      <c r="C4" s="2">
+        <v>44531</v>
       </c>
       <c r="D4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D5" t="s">
-        <v>57</v>
+        <v>56</v>
+      </c>
+      <c r="I4" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -3452,10 +3455,17 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1DE1DB4-04E1-4880-8796-F64698602DF4}">
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="16.26953125" customWidth="1"/>
+    <col min="4" max="4" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.453125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -3463,27 +3473,30 @@
         <v>8</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>12</v>
       </c>
       <c r="B2">
         <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>70</v>
       </c>
       <c r="E2">
         <v>2.6059999999999999</v>
@@ -3491,13 +3504,19 @@
       <c r="F2">
         <v>14.79</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G2">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>12</v>
       </c>
       <c r="B3">
         <v>1.5</v>
+      </c>
+      <c r="D3" t="s">
+        <v>70</v>
       </c>
       <c r="E3">
         <v>2.5619999999999998</v>
@@ -3505,13 +3524,19 @@
       <c r="F3">
         <v>16.21</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G3">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>12</v>
       </c>
       <c r="B4">
         <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>70</v>
       </c>
       <c r="E4">
         <v>2.484</v>
@@ -3519,113 +3544,136 @@
       <c r="F4">
         <v>15.45</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G4">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="B5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="D5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="B6">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E6">
+        <v>2.5720000000000001</v>
+      </c>
+      <c r="F6">
+        <v>3.39</v>
+      </c>
+      <c r="G6">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="B7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1.5</v>
+      </c>
+      <c r="D7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E7">
+        <v>2.552</v>
+      </c>
+      <c r="F7">
+        <v>5.3</v>
+      </c>
+      <c r="G7">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="D8" t="s">
+        <v>70</v>
       </c>
       <c r="E8">
-        <v>2.5720000000000001</v>
+        <v>2.5070000000000001</v>
       </c>
       <c r="F8">
-        <v>3.39</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>6.19</v>
+      </c>
+      <c r="G8">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B9">
-        <v>1.5</v>
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>70</v>
       </c>
       <c r="E9">
-        <v>2.552</v>
+        <v>2.63</v>
       </c>
       <c r="F9">
-        <v>5.3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>9.69</v>
+      </c>
+      <c r="G9">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B10">
-        <v>2</v>
+        <v>1.5</v>
+      </c>
+      <c r="D10" t="s">
+        <v>70</v>
       </c>
       <c r="E10">
-        <v>2.5070000000000001</v>
+        <v>2.6040000000000001</v>
       </c>
       <c r="F10">
-        <v>6.19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>14</v>
-      </c>
+        <v>8.57</v>
+      </c>
+      <c r="G10">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B11">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="D11" t="s">
+        <v>70</v>
       </c>
       <c r="E11">
-        <v>2.63</v>
+        <v>2.625</v>
       </c>
       <c r="F11">
-        <v>9.69</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12">
-        <v>1.5</v>
-      </c>
-      <c r="E12">
-        <v>2.6040000000000001</v>
-      </c>
-      <c r="F12">
-        <v>8.57</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13">
-        <v>2</v>
-      </c>
-      <c r="E13">
-        <v>2.625</v>
-      </c>
-      <c r="F13">
         <v>9.41</v>
+      </c>
+      <c r="G11">
+        <v>0.19</v>
       </c>
     </row>
   </sheetData>
@@ -3636,38 +3684,42 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40A95B57-D128-4B43-B63D-D25389C1CEC4}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.54296875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B3" t="s">
         <v>67</v>
       </c>
-      <c r="B2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -3678,14 +3730,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D73"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.7265625" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="21.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -3699,7 +3752,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -3713,7 +3766,7 @@
         <v>10.76</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -3727,7 +3780,7 @@
         <v>12.22</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -3741,7 +3794,7 @@
         <v>13.69</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -3755,7 +3808,7 @@
         <v>15.16</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -3769,7 +3822,7 @@
         <v>17.600000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -3783,7 +3836,7 @@
         <v>21.03</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -3797,7 +3850,7 @@
         <v>24.94</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -3811,7 +3864,7 @@
         <v>28.85</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -3825,7 +3878,7 @@
         <v>31.29</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -3839,7 +3892,7 @@
         <v>37.99</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -3853,7 +3906,7 @@
         <v>31.45</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -3867,7 +3920,7 @@
         <v>33.229999999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -3881,7 +3934,7 @@
         <v>36.450000000000003</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -3895,7 +3948,7 @@
         <v>39.03</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>12</v>
       </c>
@@ -3909,7 +3962,7 @@
         <v>41.45</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>12</v>
       </c>
@@ -3923,7 +3976,7 @@
         <v>44.35</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>12</v>
       </c>
@@ -3937,7 +3990,7 @@
         <v>46.77</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>12</v>
       </c>
@@ -3951,7 +4004,7 @@
         <v>50.58</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -3965,7 +4018,7 @@
         <v>33.369999999999997</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>12</v>
       </c>
@@ -3979,7 +4032,7 @@
         <v>36.97</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>12</v>
       </c>
@@ -3993,7 +4046,7 @@
         <v>40.58</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>12</v>
       </c>
@@ -4007,7 +4060,7 @@
         <v>43.23</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>12</v>
       </c>
@@ -4021,7 +4074,7 @@
         <v>45.09</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -4035,7 +4088,7 @@
         <v>50.24</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>13</v>
       </c>
@@ -4049,7 +4102,7 @@
         <v>21.68</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>13</v>
       </c>
@@ -4063,7 +4116,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>13</v>
       </c>
@@ -4077,7 +4130,7 @@
         <v>27.64</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>13</v>
       </c>
@@ -4091,7 +4144,7 @@
         <v>32.01</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>13</v>
       </c>
@@ -4105,7 +4158,7 @@
         <v>36.369999999999997</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>13</v>
       </c>
@@ -4119,7 +4172,7 @@
         <v>40.01</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>13</v>
       </c>
@@ -4133,7 +4186,7 @@
         <v>42.82</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>13</v>
       </c>
@@ -4147,7 +4200,7 @@
         <v>47.9</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>13</v>
       </c>
@@ -4161,7 +4214,7 @@
         <v>21.82</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>13</v>
       </c>
@@ -4175,7 +4228,7 @@
         <v>25.6</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>13</v>
       </c>
@@ -4189,7 +4242,7 @@
         <v>32.729999999999997</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>13</v>
       </c>
@@ -4203,7 +4256,7 @@
         <v>37.85</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>13</v>
       </c>
@@ -4217,7 +4270,7 @@
         <v>42.08</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>13</v>
       </c>
@@ -4231,7 +4284,7 @@
         <v>45.64</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>13</v>
       </c>
@@ -4245,7 +4298,7 @@
         <v>48.98</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>13</v>
       </c>
@@ -4259,7 +4312,7 @@
         <v>55.02</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>13</v>
       </c>
@@ -4273,7 +4326,7 @@
         <v>38.18</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>13</v>
       </c>
@@ -4287,7 +4340,7 @@
         <v>41.2</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>13</v>
       </c>
@@ -4301,7 +4354,7 @@
         <v>46.22</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>13</v>
       </c>
@@ -4315,7 +4368,7 @@
         <v>48.83</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>13</v>
       </c>
@@ -4329,7 +4382,7 @@
         <v>52.25</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>13</v>
       </c>
@@ -4343,7 +4396,7 @@
         <v>56.27</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>13</v>
       </c>
@@ -4357,7 +4410,7 @@
         <v>59.28</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>13</v>
       </c>
@@ -4371,7 +4424,7 @@
         <v>62.89</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>14</v>
       </c>
@@ -4385,7 +4438,7 @@
         <v>30.71</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>14</v>
       </c>
@@ -4399,7 +4452,7 @@
         <v>31.91</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>14</v>
       </c>
@@ -4413,7 +4466,7 @@
         <v>33.700000000000003</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>14</v>
       </c>
@@ -4427,7 +4480,7 @@
         <v>35.76</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>14</v>
       </c>
@@ -4441,7 +4494,7 @@
         <v>37.82</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>14</v>
       </c>
@@ -4455,7 +4508,7 @@
         <v>39.47</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>14</v>
       </c>
@@ -4469,7 +4522,7 @@
         <v>40.57</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>14</v>
       </c>
@@ -4483,7 +4536,7 @@
         <v>45.89</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>14</v>
       </c>
@@ -4497,7 +4550,7 @@
         <v>26.56</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>14</v>
       </c>
@@ -4511,7 +4564,7 @@
         <v>27.99</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>14</v>
       </c>
@@ -4525,7 +4578,7 @@
         <v>30.41</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>14</v>
       </c>
@@ -4539,7 +4592,7 @@
         <v>33.409999999999997</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>14</v>
       </c>
@@ -4553,7 +4606,7 @@
         <v>36.409999999999997</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>14</v>
       </c>
@@ -4567,7 +4620,7 @@
         <v>38.979999999999997</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>14</v>
       </c>
@@ -4581,7 +4634,7 @@
         <v>41.27</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>14</v>
       </c>
@@ -4595,7 +4648,7 @@
         <v>44.68</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>14</v>
       </c>
@@ -4609,7 +4662,7 @@
         <v>26.33</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>14</v>
       </c>
@@ -4623,7 +4676,7 @@
         <v>28.28</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>14</v>
       </c>
@@ -4637,7 +4690,7 @@
         <v>32.18</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>14</v>
       </c>
@@ -4651,7 +4704,7 @@
         <v>37.06</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>14</v>
       </c>
@@ -4665,7 +4718,7 @@
         <v>42.33</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>14</v>
       </c>
@@ -4679,7 +4732,7 @@
         <v>46.62</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>14</v>
       </c>
@@ -4693,7 +4746,7 @@
         <v>49.54</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>14</v>
       </c>
@@ -4715,16 +4768,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="77.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.54296875" customWidth="1"/>
+    <col min="5" max="5" width="80.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -4741,7 +4794,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -4758,7 +4811,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -4775,7 +4828,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -4799,14 +4852,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCDF4F17-6B21-47B3-8DC6-6D614FCD1B63}">
-  <dimension ref="A1:J10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="3" width="14" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="14" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="17.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4820,25 +4874,16 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>0.08</v>
       </c>
@@ -4852,25 +4897,16 @@
         <v>50.24</v>
       </c>
       <c r="E2">
-        <v>45.89</v>
+        <v>47.9</v>
       </c>
       <c r="F2">
-        <v>44.68</v>
+        <v>55.02</v>
       </c>
       <c r="G2">
-        <v>53.1</v>
-      </c>
-      <c r="H2">
-        <v>47.9</v>
-      </c>
-      <c r="I2">
-        <v>55.02</v>
-      </c>
-      <c r="J2">
         <v>62.89</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>0.16</v>
       </c>
@@ -4884,25 +4920,16 @@
         <v>58.74</v>
       </c>
       <c r="E3">
-        <v>52.24</v>
+        <v>58.7</v>
       </c>
       <c r="F3">
-        <v>51.32</v>
+        <v>65.41</v>
       </c>
       <c r="G3">
-        <v>58.95</v>
-      </c>
-      <c r="H3">
-        <v>58.7</v>
-      </c>
-      <c r="I3">
-        <v>65.41</v>
-      </c>
-      <c r="J3">
         <v>71.569999999999993</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>0.32</v>
       </c>
@@ -4916,25 +4943,16 @@
         <v>75.180000000000007</v>
       </c>
       <c r="E4">
-        <v>71.64</v>
+        <v>76.510000000000005</v>
       </c>
       <c r="F4">
-        <v>71.53</v>
+        <v>82.14</v>
       </c>
       <c r="G4">
-        <v>75.19</v>
-      </c>
-      <c r="H4">
-        <v>76.510000000000005</v>
-      </c>
-      <c r="I4">
-        <v>82.14</v>
-      </c>
-      <c r="J4">
         <v>84.77</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>0.63</v>
       </c>
@@ -4948,25 +4966,16 @@
         <v>91.68</v>
       </c>
       <c r="E5">
-        <v>91.92</v>
+        <v>91.43</v>
       </c>
       <c r="F5">
-        <v>92.58</v>
+        <v>94.92</v>
       </c>
       <c r="G5">
-        <v>93.1</v>
-      </c>
-      <c r="H5">
-        <v>91.43</v>
-      </c>
-      <c r="I5">
-        <v>94.92</v>
-      </c>
-      <c r="J5">
         <v>95.03</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1.25</v>
       </c>
@@ -4980,25 +4989,16 @@
         <v>98.85</v>
       </c>
       <c r="E6">
-        <v>99.48</v>
+        <v>97.4</v>
       </c>
       <c r="F6">
-        <v>99.6</v>
+        <v>99.04</v>
       </c>
       <c r="G6">
-        <v>99.53</v>
-      </c>
-      <c r="H6">
-        <v>97.4</v>
-      </c>
-      <c r="I6">
-        <v>99.04</v>
-      </c>
-      <c r="J6">
         <v>98.43</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>2.5</v>
       </c>
@@ -5012,25 +5012,16 @@
         <v>99.92</v>
       </c>
       <c r="E7">
-        <v>99.93</v>
+        <v>98.43</v>
       </c>
       <c r="F7">
-        <v>100</v>
+        <v>99.7</v>
       </c>
       <c r="G7">
-        <v>99.99</v>
-      </c>
-      <c r="H7">
-        <v>98.43</v>
-      </c>
-      <c r="I7">
-        <v>99.7</v>
-      </c>
-      <c r="J7">
         <v>99.3</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>5</v>
       </c>
@@ -5044,25 +5035,16 @@
         <v>100</v>
       </c>
       <c r="E8">
-        <v>100</v>
+        <v>98.9</v>
       </c>
       <c r="F8">
-        <v>100</v>
+        <v>99.8</v>
       </c>
       <c r="G8">
-        <v>100</v>
-      </c>
-      <c r="H8">
-        <v>98.9</v>
-      </c>
-      <c r="I8">
-        <v>99.8</v>
-      </c>
-      <c r="J8">
         <v>99.52</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>10</v>
       </c>
@@ -5084,17 +5066,8 @@
       <c r="G9">
         <v>100</v>
       </c>
-      <c r="H9">
-        <v>100</v>
-      </c>
-      <c r="I9">
-        <v>100</v>
-      </c>
-      <c r="J9">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>12.5</v>
       </c>
@@ -5114,15 +5087,6 @@
         <v>100</v>
       </c>
       <c r="G10">
-        <v>100</v>
-      </c>
-      <c r="H10">
-        <v>100</v>
-      </c>
-      <c r="I10">
-        <v>100</v>
-      </c>
-      <c r="J10">
         <v>100</v>
       </c>
     </row>
@@ -5134,9 +5098,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E09CC966-23FA-4723-B704-FE4E8B878F28}">
   <dimension ref="A1:J52"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="9.26953125" customWidth="1"/>
+    <col min="2" max="4" width="14" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5168,7 +5138,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1.2999999999999999E-3</v>
       </c>
@@ -5176,7 +5146,7 @@
         <v>27.64</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1.4E-3</v>
       </c>
@@ -5190,7 +5160,7 @@
         <v>28.13</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1.5E-3</v>
       </c>
@@ -5207,7 +5177,7 @@
         <v>14.11</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1.6000000000000001E-3</v>
       </c>
@@ -5215,7 +5185,7 @@
         <v>10.02</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>3.5999999999999999E-3</v>
       </c>
@@ -5223,7 +5193,7 @@
         <v>28.61</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>3.7000000000000002E-3</v>
       </c>
@@ -5231,7 +5201,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>3.8E-3</v>
       </c>
@@ -5242,7 +5212,7 @@
         <v>33.76</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>4.0000000000000001E-3</v>
       </c>
@@ -5259,7 +5229,7 @@
         <v>18.91</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>4.3E-3</v>
       </c>
@@ -5267,7 +5237,7 @@
         <v>30.71</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>4.4999999999999997E-3</v>
       </c>
@@ -5275,7 +5245,7 @@
         <v>16.7</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>4.5999999999999999E-3</v>
       </c>
@@ -5289,7 +5259,7 @@
         <v>38.18</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>4.7999999999999996E-3</v>
       </c>
@@ -5303,7 +5273,7 @@
         <v>21.68</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>4.8999999999999998E-3</v>
       </c>
@@ -5311,7 +5281,7 @@
         <v>26.33</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>5.0000000000000001E-3</v>
       </c>
@@ -5319,7 +5289,7 @@
         <v>21.82</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>6.8999999999999999E-3</v>
       </c>
@@ -5327,7 +5297,7 @@
         <v>31.91</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>7.1000000000000004E-3</v>
       </c>
@@ -5335,7 +5305,7 @@
         <v>33.229999999999997</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>7.1999999999999998E-3</v>
       </c>
@@ -5346,7 +5316,7 @@
         <v>41.2</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>7.4999999999999997E-3</v>
       </c>
@@ -5354,7 +5324,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>7.6E-3</v>
       </c>
@@ -5365,7 +5335,7 @@
         <v>28.86</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>7.7000000000000002E-3</v>
       </c>
@@ -5373,7 +5343,7 @@
         <v>28.28</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>8.0000000000000002E-3</v>
       </c>
@@ -5381,7 +5351,7 @@
         <v>25.6</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>1.2E-2</v>
       </c>
@@ -5398,7 +5368,7 @@
         <v>46.22</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>1.2800000000000001E-2</v>
       </c>
@@ -5406,7 +5376,7 @@
         <v>27.64</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>1.2999999999999999E-2</v>
       </c>
@@ -5420,7 +5390,7 @@
         <v>32.18</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>1.4E-2</v>
       </c>
@@ -5428,7 +5398,7 @@
         <v>32.729999999999997</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>1.9300000000000001E-2</v>
       </c>
@@ -5436,7 +5406,7 @@
         <v>35.76</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>0.02</v>
       </c>
@@ -5450,7 +5420,7 @@
         <v>48.83</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>2.0299999999999999E-2</v>
       </c>
@@ -5458,7 +5428,7 @@
         <v>32.01</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>2.0500000000000001E-2</v>
       </c>
@@ -5466,7 +5436,7 @@
         <v>21.03</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>2.1000000000000001E-2</v>
       </c>
@@ -5474,7 +5444,7 @@
         <v>36.97</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>2.18E-2</v>
       </c>
@@ -5482,7 +5452,7 @@
         <v>37.06</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>2.2800000000000001E-2</v>
       </c>
@@ -5490,7 +5460,7 @@
         <v>37.85</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>3.0499999999999999E-2</v>
       </c>
@@ -5498,7 +5468,7 @@
         <v>37.82</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>3.15E-2</v>
       </c>
@@ -5512,7 +5482,7 @@
         <v>52.25</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>3.1800000000000002E-2</v>
       </c>
@@ -5523,7 +5493,7 @@
         <v>36.369999999999997</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>3.3000000000000002E-2</v>
       </c>
@@ -5531,7 +5501,7 @@
         <v>40.58</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>3.3500000000000002E-2</v>
       </c>
@@ -5539,7 +5509,7 @@
         <v>42.33</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>3.4799999999999998E-2</v>
       </c>
@@ -5547,7 +5517,7 @@
         <v>42.08</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>3.95E-2</v>
       </c>
@@ -5555,7 +5525,7 @@
         <v>28.85</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>0.04</v>
       </c>
@@ -5563,7 +5533,7 @@
         <v>39.47</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>4.1000000000000002E-2</v>
       </c>
@@ -5577,7 +5547,7 @@
         <v>56.27</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>4.1500000000000002E-2</v>
       </c>
@@ -5585,7 +5555,7 @@
         <v>44.35</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>4.4499999999999998E-2</v>
       </c>
@@ -5596,7 +5566,7 @@
         <v>46.62</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>4.7E-2</v>
       </c>
@@ -5604,7 +5574,7 @@
         <v>45.64</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>5.2499999999999998E-2</v>
       </c>
@@ -5612,7 +5582,7 @@
         <v>31.29</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>5.5500000000000001E-2</v>
       </c>
@@ -5623,7 +5593,7 @@
         <v>42.92</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>5.6300000000000003E-2</v>
       </c>
@@ -5634,7 +5604,7 @@
         <v>59.28</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>5.7000000000000002E-2</v>
       </c>
@@ -5642,7 +5612,7 @@
         <v>46.77</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>6.1499999999999999E-2</v>
       </c>
@@ -5650,7 +5620,7 @@
         <v>49.54</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>6.2300000000000001E-2</v>
       </c>
@@ -5658,7 +5628,7 @@
         <v>45.09</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>6.6500000000000004E-2</v>
       </c>
@@ -5674,12 +5644,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0836405F-9CF5-4281-913C-E8A77AA637CE}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -5687,16 +5658,16 @@
         <v>8</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -5713,7 +5684,7 @@
         <v>7.72</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -5730,7 +5701,7 @@
         <v>23.32</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -5747,7 +5718,7 @@
         <v>19.14</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -5764,7 +5735,7 @@
         <v>17.36</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -5781,7 +5752,7 @@
         <v>27.79</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -5798,7 +5769,7 @@
         <v>25.45</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -5815,7 +5786,7 @@
         <v>17.440000000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -5832,7 +5803,7 @@
         <v>14.82</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -5857,9 +5828,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3CCE6D1-E56D-4E14-99BA-824197377028}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.26953125" customWidth="1"/>
+    <col min="4" max="4" width="33.1796875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -5867,27 +5843,27 @@
         <v>8</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -5898,10 +5874,10 @@
         <v>3.33</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -5912,10 +5888,10 @@
         <v>3.33</v>
       </c>
       <c r="D4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -5926,10 +5902,10 @@
         <v>3.33</v>
       </c>
       <c r="D5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -5940,10 +5916,10 @@
         <v>3.33</v>
       </c>
       <c r="D6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -5954,10 +5930,10 @@
         <v>4</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -5968,10 +5944,10 @@
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -5982,10 +5958,10 @@
         <v>2</v>
       </c>
       <c r="D9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -5996,7 +5972,7 @@
         <v>2.33</v>
       </c>
       <c r="D10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -6007,9 +5983,15 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85834437-A619-4B30-849B-1129F300A6D5}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.7265625" customWidth="1"/>
+    <col min="2" max="2" width="12.26953125" customWidth="1"/>
+    <col min="3" max="3" width="12.453125" customWidth="1"/>
+    <col min="4" max="4" width="13.1796875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -6017,13 +5999,13 @@
         <v>8</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -6037,7 +6019,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -6051,7 +6033,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -6065,7 +6047,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -6079,7 +6061,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -6093,7 +6075,7 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -6107,7 +6089,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -6121,7 +6103,7 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -6135,7 +6117,7 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -6157,9 +6139,15 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4261BF2-5CAC-49A2-AFCE-7DDA17405973}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.7265625" customWidth="1"/>
+    <col min="4" max="4" width="34.54296875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -6167,136 +6155,136 @@
         <v>8</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>44</v>
       </c>
-      <c r="D2" t="s">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3">
+        <v>1.5</v>
+      </c>
+      <c r="C3" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3">
-        <v>1.5</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6">
+        <v>1.5</v>
+      </c>
+      <c r="C6" t="s">
         <v>46</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4">
-        <v>2</v>
-      </c>
-      <c r="C4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="D7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="D8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9">
+        <v>1.5</v>
+      </c>
+      <c r="C9" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6">
-        <v>1.5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="D9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7">
-        <v>2</v>
-      </c>
-      <c r="C7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D7" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8" t="s">
-        <v>46</v>
-      </c>
-      <c r="D8" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9">
-        <v>1.5</v>
-      </c>
-      <c r="C9" t="s">
-        <v>46</v>
-      </c>
-      <c r="D9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10">
-        <v>2</v>
-      </c>
-      <c r="C10" t="s">
-        <v>46</v>
-      </c>
       <c r="D10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>